<commit_message>
Update pca with new material project phonon data for Debye temperature
</commit_message>
<xml_diff>
--- a/pca-interpretable-clustering/classified_data/Boride.xlsx
+++ b/pca-interpretable-clustering/classified_data/Boride.xlsx
@@ -2934,7 +2934,7 @@
         <v>400.90456</v>
       </c>
       <c r="H2">
-        <v>1348.90273</v>
+        <v>1348.902729</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -2960,7 +2960,7 @@
         <v>98.08154</v>
       </c>
       <c r="H3">
-        <v>649.22435</v>
+        <v>649.2243472</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -2986,7 +2986,7 @@
         <v>170.47165</v>
       </c>
       <c r="H4">
-        <v>428.78305</v>
+        <v>428.7830486</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -3012,7 +3012,7 @@
         <v>32.24355</v>
       </c>
       <c r="H5">
-        <v>292.63442</v>
+        <v>292.6344243</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -3038,7 +3038,7 @@
         <v>106.21901</v>
       </c>
       <c r="H6">
-        <v>713.72609</v>
+        <v>713.7260923</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -3064,7 +3064,7 @@
         <v>15.32444</v>
       </c>
       <c r="H7">
-        <v>347.39582</v>
+        <v>347.3958166</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -3090,7 +3090,7 @@
         <v>63.33309</v>
       </c>
       <c r="H8">
-        <v>470.14881</v>
+        <v>470.1488106</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -3116,7 +3116,7 @@
         <v>14.95567</v>
       </c>
       <c r="H9">
-        <v>118.72315</v>
+        <v>118.7231493</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -3142,7 +3142,7 @@
         <v>21.01009</v>
       </c>
       <c r="H10">
-        <v>228.75884</v>
+        <v>228.7588424</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -3168,7 +3168,7 @@
         <v>301.39574</v>
       </c>
       <c r="H11">
-        <v>472.34063</v>
+        <v>472.3406349</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -3194,7 +3194,7 @@
         <v>17.23168</v>
       </c>
       <c r="H12">
-        <v>144.49243</v>
+        <v>144.4924293</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -3220,7 +3220,7 @@
         <v>494.27215</v>
       </c>
       <c r="H13">
-        <v>616.68553</v>
+        <v>616.6855276</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -3246,7 +3246,7 @@
         <v>228.79363</v>
       </c>
       <c r="H14">
-        <v>892.88072</v>
+        <v>892.8807197</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -3272,7 +3272,7 @@
         <v>59.32077</v>
       </c>
       <c r="H15">
-        <v>289.75051</v>
+        <v>289.7505118</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -3298,7 +3298,7 @@
         <v>201.63311</v>
       </c>
       <c r="H16">
-        <v>775.99955</v>
+        <v>775.999554</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -3324,7 +3324,7 @@
         <v>465.96092</v>
       </c>
       <c r="H17">
-        <v>605.88208</v>
+        <v>605.882078</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -3350,7 +3350,7 @@
         <v>198.59808</v>
       </c>
       <c r="H18">
-        <v>334.13285</v>
+        <v>334.1328488</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -3376,7 +3376,7 @@
         <v>180.45822</v>
       </c>
       <c r="H19">
-        <v>341.11889</v>
+        <v>341.1188852</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -3402,7 +3402,7 @@
         <v>440.45883</v>
       </c>
       <c r="H20">
-        <v>931.16047</v>
+        <v>931.1604677</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -3428,7 +3428,7 @@
         <v>359.80614</v>
       </c>
       <c r="H21">
-        <v>722.00472</v>
+        <v>722.004717</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -3454,7 +3454,7 @@
         <v>414.36685</v>
       </c>
       <c r="H22">
-        <v>716.60381</v>
+        <v>716.6038138</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -3480,7 +3480,7 @@
         <v>460.62438</v>
       </c>
       <c r="H23">
-        <v>1093.70463</v>
+        <v>1093.704625</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -3506,7 +3506,7 @@
         <v>455.60121</v>
       </c>
       <c r="H24">
-        <v>844.18483</v>
+        <v>844.1848282</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -3532,7 +3532,7 @@
         <v>411.74725</v>
       </c>
       <c r="H25">
-        <v>968.98297</v>
+        <v>968.9829745</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -3558,7 +3558,7 @@
         <v>359.31787</v>
       </c>
       <c r="H26">
-        <v>732.51458</v>
+        <v>732.5145782</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -3584,7 +3584,7 @@
         <v>127.67544</v>
       </c>
       <c r="H27">
-        <v>315.3074</v>
+        <v>315.3074013</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -3610,7 +3610,7 @@
         <v>596.12769</v>
       </c>
       <c r="H28">
-        <v>1310.97645</v>
+        <v>1310.976454</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -3636,7 +3636,7 @@
         <v>561.65316</v>
       </c>
       <c r="H29">
-        <v>1242.22572</v>
+        <v>1242.225724</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -3688,7 +3688,7 @@
         <v>426.00392</v>
       </c>
       <c r="H31">
-        <v>756.66507</v>
+        <v>756.6650719</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -3714,7 +3714,7 @@
         <v>56.09652</v>
       </c>
       <c r="H32">
-        <v>322.97722</v>
+        <v>322.9772171</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -3740,7 +3740,7 @@
         <v>110.10008</v>
       </c>
       <c r="H33">
-        <v>392.28834</v>
+        <v>392.2883405</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -3766,7 +3766,7 @@
         <v>385.94366</v>
       </c>
       <c r="H34">
-        <v>750.73994</v>
+        <v>750.7399421</v>
       </c>
     </row>
     <row r="35" spans="1:8">
@@ -3792,7 +3792,7 @@
         <v>487.73252</v>
       </c>
       <c r="H35">
-        <v>574.94192</v>
+        <v>574.9419185</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -3844,7 +3844,7 @@
         <v>47.94118</v>
       </c>
       <c r="H37">
-        <v>421.45162</v>
+        <v>421.4516237</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -3870,7 +3870,7 @@
         <v>218.12679</v>
       </c>
       <c r="H38">
-        <v>498.96617</v>
+        <v>498.9661706</v>
       </c>
     </row>
     <row r="39" spans="1:8">
@@ -3896,7 +3896,7 @@
         <v>21.93246</v>
       </c>
       <c r="H39">
-        <v>223.75363</v>
+        <v>223.7536286</v>
       </c>
     </row>
     <row r="40" spans="1:8">
@@ -3922,7 +3922,7 @@
         <v>437.6727</v>
       </c>
       <c r="H40">
-        <v>959.55565</v>
+        <v>959.5556475</v>
       </c>
     </row>
     <row r="41" spans="1:8">
@@ -3948,7 +3948,7 @@
         <v>333.0004</v>
       </c>
       <c r="H41">
-        <v>671.01061</v>
+        <v>671.0106122</v>
       </c>
     </row>
     <row r="42" spans="1:8">
@@ -3974,7 +3974,7 @@
         <v>507.1632</v>
       </c>
       <c r="H42">
-        <v>564.29991</v>
+        <v>564.2999135</v>
       </c>
     </row>
     <row r="43" spans="1:8">
@@ -4000,7 +4000,7 @@
         <v>394.16803</v>
       </c>
       <c r="H43">
-        <v>792.21857</v>
+        <v>792.2185692</v>
       </c>
     </row>
     <row r="44" spans="1:8">
@@ -4026,7 +4026,7 @@
         <v>32.37439</v>
       </c>
       <c r="H44">
-        <v>323.8999</v>
+        <v>323.8998963</v>
       </c>
     </row>
     <row r="45" spans="1:8">
@@ -4052,7 +4052,7 @@
         <v>475.2672</v>
       </c>
       <c r="H45">
-        <v>749.65872</v>
+        <v>749.6587227</v>
       </c>
     </row>
     <row r="46" spans="1:8">
@@ -4078,7 +4078,7 @@
         <v>510.86683</v>
       </c>
       <c r="H46">
-        <v>569.79045</v>
+        <v>569.7904507</v>
       </c>
     </row>
     <row r="47" spans="1:8">
@@ -4104,7 +4104,7 @@
         <v>560.07178</v>
       </c>
       <c r="H47">
-        <v>1082.3994</v>
+        <v>1082.399398</v>
       </c>
     </row>
     <row r="48" spans="1:8">
@@ -4130,7 +4130,7 @@
         <v>540.5413600000001</v>
       </c>
       <c r="H48">
-        <v>1006.6157</v>
+        <v>1006.615696</v>
       </c>
     </row>
     <row r="49" spans="1:8">
@@ -4156,7 +4156,7 @@
         <v>496.55872</v>
       </c>
       <c r="H49">
-        <v>963.29701</v>
+        <v>963.2970091</v>
       </c>
     </row>
     <row r="50" spans="1:8">
@@ -4182,7 +4182,7 @@
         <v>423.43144</v>
       </c>
       <c r="H50">
-        <v>895.36126</v>
+        <v>895.3612616</v>
       </c>
     </row>
     <row r="51" spans="1:8">
@@ -4208,7 +4208,7 @@
         <v>333.27489</v>
       </c>
       <c r="H51">
-        <v>756.43506</v>
+        <v>756.4350586</v>
       </c>
     </row>
     <row r="52" spans="1:8">
@@ -4234,7 +4234,7 @@
         <v>336.91231</v>
       </c>
       <c r="H52">
-        <v>615.46704</v>
+        <v>615.4670434</v>
       </c>
     </row>
     <row r="53" spans="1:8">
@@ -4260,7 +4260,7 @@
         <v>343.37168</v>
       </c>
       <c r="H53">
-        <v>610.0835</v>
+        <v>610.0834963</v>
       </c>
     </row>
     <row r="54" spans="1:8">
@@ -4286,7 +4286,7 @@
         <v>370.16845</v>
       </c>
       <c r="H54">
-        <v>814.77135</v>
+        <v>814.771354</v>
       </c>
     </row>
     <row r="55" spans="1:8">
@@ -4312,7 +4312,7 @@
         <v>497.82924</v>
       </c>
       <c r="H55">
-        <v>579.0787</v>
+        <v>579.0787048</v>
       </c>
     </row>
     <row r="56" spans="1:8">
@@ -4338,7 +4338,7 @@
         <v>290.01764</v>
       </c>
       <c r="H56">
-        <v>565.5875</v>
+        <v>565.5874964</v>
       </c>
     </row>
     <row r="57" spans="1:8">
@@ -4364,7 +4364,7 @@
         <v>509.92399</v>
       </c>
       <c r="H57">
-        <v>622.42683</v>
+        <v>622.4268315</v>
       </c>
     </row>
     <row r="58" spans="1:8">
@@ -4390,7 +4390,7 @@
         <v>545.5519399999999</v>
       </c>
       <c r="H58">
-        <v>1033.50716</v>
+        <v>1033.507162</v>
       </c>
     </row>
     <row r="59" spans="1:8">
@@ -4416,7 +4416,7 @@
         <v>12.19056</v>
       </c>
       <c r="H59">
-        <v>317.48209</v>
+        <v>317.4820943</v>
       </c>
     </row>
     <row r="60" spans="1:8">
@@ -4442,7 +4442,7 @@
         <v>140.96945</v>
       </c>
       <c r="H60">
-        <v>402.05329</v>
+        <v>402.053291</v>
       </c>
     </row>
     <row r="61" spans="1:8">
@@ -4468,7 +4468,7 @@
         <v>182.6933</v>
       </c>
       <c r="H61">
-        <v>392.60609</v>
+        <v>392.6060907</v>
       </c>
     </row>
     <row r="62" spans="1:8">
@@ -4494,7 +4494,7 @@
         <v>178.2848</v>
       </c>
       <c r="H62">
-        <v>338.09261</v>
+        <v>338.0926128</v>
       </c>
     </row>
     <row r="63" spans="1:8">
@@ -4520,7 +4520,7 @@
         <v>122.4292</v>
       </c>
       <c r="H63">
-        <v>272.68295</v>
+        <v>272.6829454</v>
       </c>
     </row>
     <row r="64" spans="1:8">
@@ -4546,7 +4546,7 @@
         <v>517.36146</v>
       </c>
       <c r="H64">
-        <v>576.81942</v>
+        <v>576.8194218</v>
       </c>
     </row>
     <row r="65" spans="1:8">
@@ -4572,7 +4572,7 @@
         <v>521.5513</v>
       </c>
       <c r="H65">
-        <v>763.41216</v>
+        <v>763.4121613</v>
       </c>
     </row>
     <row r="66" spans="1:8">
@@ -4598,7 +4598,7 @@
         <v>475.40034</v>
       </c>
       <c r="H66">
-        <v>781.9032099999999</v>
+        <v>781.9032121</v>
       </c>
     </row>
     <row r="67" spans="1:8">
@@ -4624,7 +4624,7 @@
         <v>449.89798</v>
       </c>
       <c r="H67">
-        <v>688.0032</v>
+        <v>688.0032001</v>
       </c>
     </row>
     <row r="68" spans="1:8">
@@ -4650,7 +4650,7 @@
         <v>507.77467</v>
       </c>
       <c r="H68">
-        <v>597.4299600000001</v>
+        <v>597.429964</v>
       </c>
     </row>
     <row r="69" spans="1:8">
@@ -4676,7 +4676,7 @@
         <v>493.96586</v>
       </c>
       <c r="H69">
-        <v>1057.74049</v>
+        <v>1057.740486</v>
       </c>
     </row>
     <row r="70" spans="1:8">
@@ -4702,7 +4702,7 @@
         <v>441.31198</v>
       </c>
       <c r="H70">
-        <v>746.87769</v>
+        <v>746.8776867</v>
       </c>
     </row>
     <row r="71" spans="1:8">
@@ -4728,7 +4728,7 @@
         <v>548.0857999999999</v>
       </c>
       <c r="H71">
-        <v>1050.97821</v>
+        <v>1050.978208</v>
       </c>
     </row>
     <row r="72" spans="1:8">
@@ -4754,7 +4754,7 @@
         <v>426.76049</v>
       </c>
       <c r="H72">
-        <v>1435.14257</v>
+        <v>1435.142568</v>
       </c>
     </row>
     <row r="73" spans="1:8">
@@ -4780,7 +4780,7 @@
         <v>411.91425</v>
       </c>
       <c r="H73">
-        <v>1368.13307</v>
+        <v>1368.133068</v>
       </c>
     </row>
     <row r="74" spans="1:8">
@@ -4806,7 +4806,7 @@
         <v>304.33469</v>
       </c>
       <c r="H74">
-        <v>1096.7477</v>
+        <v>1096.747705</v>
       </c>
     </row>
     <row r="75" spans="1:8">
@@ -4832,7 +4832,7 @@
         <v>99.91969</v>
       </c>
       <c r="H75">
-        <v>501.57882</v>
+        <v>501.5788171</v>
       </c>
     </row>
     <row r="76" spans="1:8">
@@ -4858,7 +4858,7 @@
         <v>306.26973</v>
       </c>
       <c r="H76">
-        <v>619.94157</v>
+        <v>619.9415669</v>
       </c>
     </row>
     <row r="77" spans="1:8">
@@ -4884,7 +4884,7 @@
         <v>290.60326</v>
       </c>
       <c r="H77">
-        <v>589.64703</v>
+        <v>589.6470288</v>
       </c>
     </row>
     <row r="78" spans="1:8">
@@ -4910,7 +4910,7 @@
         <v>167.433</v>
       </c>
       <c r="H78">
-        <v>269.75852</v>
+        <v>269.7585163</v>
       </c>
     </row>
     <row r="79" spans="1:8">
@@ -4936,7 +4936,7 @@
         <v>163.55641</v>
       </c>
       <c r="H79">
-        <v>266.30552</v>
+        <v>266.3055195</v>
       </c>
     </row>
     <row r="80" spans="1:8">
@@ -4962,7 +4962,7 @@
         <v>163.41262</v>
       </c>
       <c r="H80">
-        <v>267.38878</v>
+        <v>267.3887803</v>
       </c>
     </row>
     <row r="81" spans="1:8">
@@ -4988,7 +4988,7 @@
         <v>160.94419</v>
       </c>
       <c r="H81">
-        <v>541.6889</v>
+        <v>535.6092675</v>
       </c>
     </row>
     <row r="82" spans="1:8">
@@ -5014,7 +5014,7 @@
         <v>62.61357</v>
       </c>
       <c r="H82">
-        <v>392.60419</v>
+        <v>392.6041937</v>
       </c>
     </row>
     <row r="83" spans="1:8">
@@ -5040,7 +5040,7 @@
         <v>328.78957</v>
       </c>
       <c r="H83">
-        <v>675.87805</v>
+        <v>675.878047</v>
       </c>
     </row>
     <row r="84" spans="1:8">
@@ -5066,7 +5066,7 @@
         <v>356.6311</v>
       </c>
       <c r="H84">
-        <v>782.87387</v>
+        <v>782.8738664</v>
       </c>
     </row>
     <row r="85" spans="1:8">
@@ -5092,7 +5092,7 @@
         <v>310.73625</v>
       </c>
       <c r="H85">
-        <v>639.76577</v>
+        <v>639.7657657</v>
       </c>
     </row>
     <row r="86" spans="1:8">
@@ -5118,7 +5118,7 @@
         <v>467.03055</v>
       </c>
       <c r="H86">
-        <v>554.30923</v>
+        <v>554.3092345</v>
       </c>
     </row>
     <row r="87" spans="1:8">
@@ -5144,7 +5144,7 @@
         <v>413.97886</v>
       </c>
       <c r="H87">
-        <v>658.96282</v>
+        <v>658.9628218</v>
       </c>
     </row>
     <row r="88" spans="1:8">
@@ -5170,7 +5170,7 @@
         <v>453.528</v>
       </c>
       <c r="H88">
-        <v>673.58744</v>
+        <v>673.5874357</v>
       </c>
     </row>
     <row r="89" spans="1:8">
@@ -5196,7 +5196,7 @@
         <v>331.15552</v>
       </c>
       <c r="H89">
-        <v>861.01653</v>
+        <v>861.016526</v>
       </c>
     </row>
     <row r="90" spans="1:8">
@@ -5222,7 +5222,7 @@
         <v>474.85218</v>
       </c>
       <c r="H90">
-        <v>892.1341</v>
+        <v>892.1341009</v>
       </c>
     </row>
     <row r="91" spans="1:8">
@@ -5248,7 +5248,7 @@
         <v>320.75102</v>
       </c>
       <c r="H91">
-        <v>1398.23634</v>
+        <v>1398.236336</v>
       </c>
     </row>
     <row r="92" spans="1:8">
@@ -5274,7 +5274,7 @@
         <v>184.34539</v>
       </c>
       <c r="H92">
-        <v>411.1294</v>
+        <v>411.1293984</v>
       </c>
     </row>
     <row r="93" spans="1:8">
@@ -5300,7 +5300,7 @@
         <v>27.78672</v>
       </c>
       <c r="H93">
-        <v>492.43049</v>
+        <v>492.4304851</v>
       </c>
     </row>
     <row r="94" spans="1:8">
@@ -5326,7 +5326,7 @@
         <v>158.4597</v>
       </c>
       <c r="H94">
-        <v>318.60698</v>
+        <v>389.252164</v>
       </c>
     </row>
     <row r="95" spans="1:8">
@@ -5352,7 +5352,7 @@
         <v>124.24347</v>
       </c>
       <c r="H95">
-        <v>342.1295</v>
+        <v>394.3786955</v>
       </c>
     </row>
     <row r="96" spans="1:8">
@@ -5378,7 +5378,7 @@
         <v>271.9416</v>
       </c>
       <c r="H96">
-        <v>521.21817</v>
+        <v>521.2181707</v>
       </c>
     </row>
     <row r="97" spans="1:8">
@@ -5404,7 +5404,7 @@
         <v>203.24224</v>
       </c>
       <c r="H97">
-        <v>455.28674</v>
+        <v>455.2867441</v>
       </c>
     </row>
     <row r="98" spans="1:8">
@@ -5430,7 +5430,7 @@
         <v>262.66524</v>
       </c>
       <c r="H98">
-        <v>515.3039</v>
+        <v>431.0238701</v>
       </c>
     </row>
     <row r="99" spans="1:8">
@@ -5456,7 +5456,7 @@
         <v>201.02798</v>
       </c>
       <c r="H99">
-        <v>455.93967</v>
+        <v>455.9396718</v>
       </c>
     </row>
     <row r="100" spans="1:8">
@@ -5482,7 +5482,7 @@
         <v>268.36684</v>
       </c>
       <c r="H100">
-        <v>518.59054</v>
+        <v>518.5905442</v>
       </c>
     </row>
     <row r="101" spans="1:8">
@@ -5508,7 +5508,7 @@
         <v>200.885</v>
       </c>
       <c r="H101">
-        <v>454.43542</v>
+        <v>454.435416</v>
       </c>
     </row>
     <row r="102" spans="1:8">
@@ -5534,7 +5534,7 @@
         <v>204.51297</v>
       </c>
       <c r="H102">
-        <v>481.45674</v>
+        <v>481.4567432</v>
       </c>
     </row>
     <row r="103" spans="1:8">
@@ -5560,7 +5560,7 @@
         <v>222.43485</v>
       </c>
       <c r="H103">
-        <v>496.58216</v>
+        <v>496.5821647</v>
       </c>
     </row>
     <row r="104" spans="1:8">
@@ -5586,7 +5586,7 @@
         <v>241.87531</v>
       </c>
       <c r="H104">
-        <v>506.41379</v>
+        <v>506.4137855</v>
       </c>
     </row>
     <row r="105" spans="1:8">
@@ -5612,7 +5612,7 @@
         <v>198.18842</v>
       </c>
       <c r="H105">
-        <v>455.51098</v>
+        <v>455.5109752</v>
       </c>
     </row>
     <row r="106" spans="1:8">
@@ -5638,7 +5638,7 @@
         <v>261.83155</v>
       </c>
       <c r="H106">
-        <v>592.78867</v>
+        <v>592.788673</v>
       </c>
     </row>
     <row r="107" spans="1:8">
@@ -5664,7 +5664,7 @@
         <v>200.50886</v>
       </c>
       <c r="H107">
-        <v>525.9175</v>
+        <v>525.9174972</v>
       </c>
     </row>
     <row r="108" spans="1:8">
@@ -5690,7 +5690,7 @@
         <v>275.93059</v>
       </c>
       <c r="H108">
-        <v>411.67</v>
+        <v>411.6700046</v>
       </c>
     </row>
     <row r="109" spans="1:8">
@@ -5716,7 +5716,7 @@
         <v>408.47383</v>
       </c>
       <c r="H109">
-        <v>439.44939</v>
+        <v>439.4493852</v>
       </c>
     </row>
     <row r="110" spans="1:8">
@@ -5742,7 +5742,7 @@
         <v>347.96961</v>
       </c>
       <c r="H110">
-        <v>685.6843699999999</v>
+        <v>685.6843714</v>
       </c>
     </row>
     <row r="111" spans="1:8">
@@ -5768,7 +5768,7 @@
         <v>259.45094</v>
       </c>
       <c r="H111">
-        <v>564.25792</v>
+        <v>564.2579203</v>
       </c>
     </row>
     <row r="112" spans="1:8">
@@ -5794,7 +5794,7 @@
         <v>504.85237</v>
       </c>
       <c r="H112">
-        <v>742.23245</v>
+        <v>742.2324456</v>
       </c>
     </row>
     <row r="113" spans="1:8">
@@ -5820,7 +5820,7 @@
         <v>494.90166</v>
       </c>
       <c r="H113">
-        <v>540.41049</v>
+        <v>540.4104928</v>
       </c>
     </row>
     <row r="114" spans="1:8">
@@ -5846,7 +5846,7 @@
         <v>553.2433</v>
       </c>
       <c r="H114">
-        <v>985.44946</v>
+        <v>985.4494623000001</v>
       </c>
     </row>
     <row r="115" spans="1:8">
@@ -5872,7 +5872,7 @@
         <v>356.80247</v>
       </c>
       <c r="H115">
-        <v>836.71545</v>
+        <v>836.7154518999999</v>
       </c>
     </row>
     <row r="116" spans="1:8">
@@ -5898,7 +5898,7 @@
         <v>139.19304</v>
       </c>
       <c r="H116">
-        <v>540.07712</v>
+        <v>540.0771246</v>
       </c>
     </row>
     <row r="117" spans="1:8">
@@ -5924,7 +5924,7 @@
         <v>19.34507</v>
       </c>
       <c r="H117">
-        <v>275.77611</v>
+        <v>275.7761117</v>
       </c>
     </row>
     <row r="118" spans="1:8">
@@ -5950,7 +5950,7 @@
         <v>82.53234999999999</v>
       </c>
       <c r="H118">
-        <v>435.48131</v>
+        <v>435.4813143</v>
       </c>
     </row>
     <row r="119" spans="1:8">
@@ -5976,7 +5976,7 @@
         <v>83.84712</v>
       </c>
       <c r="H119">
-        <v>551.3586299999999</v>
+        <v>551.3586311</v>
       </c>
     </row>
     <row r="120" spans="1:8">
@@ -6002,7 +6002,7 @@
         <v>85.60612</v>
       </c>
       <c r="H120">
-        <v>535.33661</v>
+        <v>535.3366116</v>
       </c>
     </row>
     <row r="121" spans="1:8">
@@ -6028,7 +6028,7 @@
         <v>513.72387</v>
       </c>
       <c r="H121">
-        <v>859.64363</v>
+        <v>859.6436348</v>
       </c>
     </row>
     <row r="122" spans="1:8">
@@ -6054,7 +6054,7 @@
         <v>129.53161</v>
       </c>
       <c r="H122">
-        <v>416.12373</v>
+        <v>339.3160091</v>
       </c>
     </row>
     <row r="123" spans="1:8">
@@ -6080,7 +6080,7 @@
         <v>86.90751</v>
       </c>
       <c r="H123">
-        <v>453.33813</v>
+        <v>453.3381308</v>
       </c>
     </row>
     <row r="124" spans="1:8">
@@ -6106,7 +6106,7 @@
         <v>368.52033</v>
       </c>
       <c r="H124">
-        <v>1269.55406</v>
+        <v>1269.554058</v>
       </c>
     </row>
     <row r="125" spans="1:8">
@@ -6132,7 +6132,7 @@
         <v>162.35835</v>
       </c>
       <c r="H125">
-        <v>512.68448</v>
+        <v>512.6844755</v>
       </c>
     </row>
     <row r="126" spans="1:8">
@@ -6158,7 +6158,7 @@
         <v>54.5532</v>
       </c>
       <c r="H126">
-        <v>436.87467</v>
+        <v>436.8746704</v>
       </c>
     </row>
     <row r="127" spans="1:8">
@@ -6184,7 +6184,7 @@
         <v>185.87637</v>
       </c>
       <c r="H127">
-        <v>705.3656</v>
+        <v>718.0103441</v>
       </c>
     </row>
     <row r="128" spans="1:8">
@@ -6210,7 +6210,7 @@
         <v>77.69414</v>
       </c>
       <c r="H128">
-        <v>312.90796</v>
+        <v>312.9079583</v>
       </c>
     </row>
     <row r="129" spans="1:8">
@@ -6236,7 +6236,7 @@
         <v>29.63808</v>
       </c>
       <c r="H129">
-        <v>149.94328</v>
+        <v>149.9432771</v>
       </c>
     </row>
     <row r="130" spans="1:8">
@@ -6262,7 +6262,7 @@
         <v>141.37323</v>
       </c>
       <c r="H130">
-        <v>271.11488</v>
+        <v>271.1148759</v>
       </c>
     </row>
     <row r="131" spans="1:8">
@@ -6288,7 +6288,7 @@
         <v>226.9409</v>
       </c>
       <c r="H131">
-        <v>582.16666</v>
+        <v>582.1666648</v>
       </c>
     </row>
     <row r="132" spans="1:8">
@@ -6314,7 +6314,7 @@
         <v>561.92851</v>
       </c>
       <c r="H132">
-        <v>678.0087</v>
+        <v>678.0087049</v>
       </c>
     </row>
     <row r="133" spans="1:8">
@@ -6340,7 +6340,7 @@
         <v>531.09735</v>
       </c>
       <c r="H133">
-        <v>551.60691</v>
+        <v>551.6069060999999</v>
       </c>
     </row>
     <row r="134" spans="1:8">
@@ -6366,7 +6366,7 @@
         <v>209.42679</v>
       </c>
       <c r="H134">
-        <v>496.64843</v>
+        <v>496.6484346</v>
       </c>
     </row>
     <row r="135" spans="1:8">
@@ -6418,7 +6418,7 @@
         <v>159.133</v>
       </c>
       <c r="H136">
-        <v>446.5609</v>
+        <v>359.3270258</v>
       </c>
     </row>
     <row r="137" spans="1:8">
@@ -6444,7 +6444,7 @@
         <v>314.86612</v>
       </c>
       <c r="H137">
-        <v>398.05512</v>
+        <v>398.0551223</v>
       </c>
     </row>
     <row r="138" spans="1:8">
@@ -6470,7 +6470,7 @@
         <v>256.83668</v>
       </c>
       <c r="H138">
-        <v>448.31521</v>
+        <v>448.3152102</v>
       </c>
     </row>
     <row r="139" spans="1:8">
@@ -6496,7 +6496,7 @@
         <v>374.25293</v>
       </c>
       <c r="H139">
-        <v>618.23762</v>
+        <v>618.2376181</v>
       </c>
     </row>
     <row r="140" spans="1:8">
@@ -6522,7 +6522,7 @@
         <v>315.53142</v>
       </c>
       <c r="H140">
-        <v>389.5011</v>
+        <v>389.5011045</v>
       </c>
     </row>
     <row r="141" spans="1:8">
@@ -6548,7 +6548,7 @@
         <v>274.16245</v>
       </c>
       <c r="H141">
-        <v>450.32431</v>
+        <v>450.3243127</v>
       </c>
     </row>
     <row r="142" spans="1:8">
@@ -6574,7 +6574,7 @@
         <v>315.49538</v>
       </c>
       <c r="H142">
-        <v>548.15412</v>
+        <v>548.1541162</v>
       </c>
     </row>
     <row r="143" spans="1:8">
@@ -6600,7 +6600,7 @@
         <v>204.65617</v>
       </c>
       <c r="H143">
-        <v>421.06489</v>
+        <v>357.6136663</v>
       </c>
     </row>
     <row r="144" spans="1:8">
@@ -6626,7 +6626,7 @@
         <v>351.8172</v>
       </c>
       <c r="H144">
-        <v>607.2591200000001</v>
+        <v>607.2591171</v>
       </c>
     </row>
     <row r="145" spans="1:8">
@@ -6652,7 +6652,7 @@
         <v>316.93662</v>
       </c>
       <c r="H145">
-        <v>392.30058</v>
+        <v>392.3005835</v>
       </c>
     </row>
     <row r="146" spans="1:8">
@@ -6678,7 +6678,7 @@
         <v>272.78986</v>
       </c>
       <c r="H146">
-        <v>451.99066</v>
+        <v>364.5200544</v>
       </c>
     </row>
     <row r="147" spans="1:8">
@@ -6704,7 +6704,7 @@
         <v>306.25422</v>
       </c>
       <c r="H147">
-        <v>544.67736</v>
+        <v>544.6773635</v>
       </c>
     </row>
     <row r="148" spans="1:8">
@@ -6730,7 +6730,7 @@
         <v>554.2062100000001</v>
       </c>
       <c r="H148">
-        <v>711.36659</v>
+        <v>711.3665885</v>
       </c>
     </row>
     <row r="149" spans="1:8">
@@ -6756,7 +6756,7 @@
         <v>539.12765</v>
       </c>
       <c r="H149">
-        <v>685.10436</v>
+        <v>685.1043639</v>
       </c>
     </row>
     <row r="150" spans="1:8">
@@ -6782,7 +6782,7 @@
         <v>363.27158</v>
       </c>
       <c r="H150">
-        <v>613.30786</v>
+        <v>613.3078647</v>
       </c>
     </row>
     <row r="151" spans="1:8">
@@ -6808,7 +6808,7 @@
         <v>311.30727</v>
       </c>
       <c r="H151">
-        <v>547.87492</v>
+        <v>547.8749213</v>
       </c>
     </row>
     <row r="152" spans="1:8">
@@ -6834,7 +6834,7 @@
         <v>202.368</v>
       </c>
       <c r="H152">
-        <v>421.60858</v>
+        <v>356.0152853</v>
       </c>
     </row>
     <row r="153" spans="1:8">
@@ -6860,7 +6860,7 @@
         <v>174.28368</v>
       </c>
       <c r="H153">
-        <v>406.55428</v>
+        <v>406.5542832</v>
       </c>
     </row>
     <row r="154" spans="1:8">
@@ -6886,7 +6886,7 @@
         <v>312.85687</v>
       </c>
       <c r="H154">
-        <v>385.12519</v>
+        <v>385.1251918</v>
       </c>
     </row>
     <row r="155" spans="1:8">
@@ -6912,7 +6912,7 @@
         <v>274.87879</v>
       </c>
       <c r="H155">
-        <v>446.57067</v>
+        <v>446.5706735</v>
       </c>
     </row>
     <row r="156" spans="1:8">
@@ -6938,7 +6938,7 @@
         <v>272.58656</v>
       </c>
       <c r="H156">
-        <v>1015.88172</v>
+        <v>1015.881725</v>
       </c>
     </row>
     <row r="157" spans="1:8">
@@ -6964,7 +6964,7 @@
         <v>96.36588</v>
       </c>
       <c r="H157">
-        <v>217.26373</v>
+        <v>217.2637286</v>
       </c>
     </row>
     <row r="158" spans="1:8">
@@ -6990,7 +6990,7 @@
         <v>489.58425</v>
       </c>
       <c r="H158">
-        <v>852.38851</v>
+        <v>852.3885122</v>
       </c>
     </row>
     <row r="159" spans="1:8">
@@ -7016,7 +7016,7 @@
         <v>235.38434</v>
       </c>
       <c r="H159">
-        <v>426.98921</v>
+        <v>426.9892059</v>
       </c>
     </row>
     <row r="160" spans="1:8">
@@ -7042,7 +7042,7 @@
         <v>183.20036</v>
       </c>
       <c r="H160">
-        <v>413.98727</v>
+        <v>413.9872678</v>
       </c>
     </row>
     <row r="161" spans="1:8">
@@ -7068,7 +7068,7 @@
         <v>254.61824</v>
       </c>
       <c r="H161">
-        <v>355.90736</v>
+        <v>355.9073583</v>
       </c>
     </row>
     <row r="162" spans="1:8">
@@ -7094,7 +7094,7 @@
         <v>437.82892</v>
       </c>
       <c r="H162">
-        <v>1104.38757</v>
+        <v>1104.387565</v>
       </c>
     </row>
     <row r="163" spans="1:8">
@@ -7120,7 +7120,7 @@
         <v>264.56865</v>
       </c>
       <c r="H163">
-        <v>451.07962</v>
+        <v>451.0796208</v>
       </c>
     </row>
     <row r="164" spans="1:8">
@@ -7146,7 +7146,7 @@
         <v>490.59288</v>
       </c>
       <c r="H164">
-        <v>637.27181</v>
+        <v>571.8139008000001</v>
       </c>
     </row>
     <row r="165" spans="1:8">
@@ -7172,7 +7172,7 @@
         <v>561.13212</v>
       </c>
       <c r="H165">
-        <v>843.97337</v>
+        <v>843.9733665</v>
       </c>
     </row>
     <row r="166" spans="1:8">
@@ -7198,7 +7198,7 @@
         <v>318.40758</v>
       </c>
       <c r="H166">
-        <v>394.58325</v>
+        <v>394.5832498</v>
       </c>
     </row>
     <row r="167" spans="1:8">
@@ -7224,7 +7224,7 @@
         <v>272.01744</v>
       </c>
       <c r="H167">
-        <v>453.25268</v>
+        <v>453.2526802</v>
       </c>
     </row>
     <row r="168" spans="1:8">
@@ -7250,7 +7250,7 @@
         <v>302.97959</v>
       </c>
       <c r="H168">
-        <v>544.43936</v>
+        <v>544.4393609</v>
       </c>
     </row>
     <row r="169" spans="1:8">
@@ -7276,7 +7276,7 @@
         <v>311.9016</v>
       </c>
       <c r="H169">
-        <v>373.96593</v>
+        <v>373.9659307</v>
       </c>
     </row>
     <row r="170" spans="1:8">
@@ -7302,7 +7302,7 @@
         <v>248.7804</v>
       </c>
       <c r="H170">
-        <v>403.40379</v>
+        <v>403.4037889</v>
       </c>
     </row>
     <row r="171" spans="1:8">
@@ -7328,7 +7328,7 @@
         <v>551.35661</v>
       </c>
       <c r="H171">
-        <v>1020.00007</v>
+        <v>1020.000071</v>
       </c>
     </row>
     <row r="172" spans="1:8">
@@ -7354,7 +7354,7 @@
         <v>376.06745</v>
       </c>
       <c r="H172">
-        <v>614.06184</v>
+        <v>614.061842</v>
       </c>
     </row>
     <row r="173" spans="1:8">
@@ -7380,7 +7380,7 @@
         <v>275.1352</v>
       </c>
       <c r="H173">
-        <v>450.09509</v>
+        <v>450.0950938</v>
       </c>
     </row>
     <row r="174" spans="1:8">
@@ -7406,7 +7406,7 @@
         <v>316.04446</v>
       </c>
       <c r="H174">
-        <v>547.57813</v>
+        <v>547.5781251</v>
       </c>
     </row>
     <row r="175" spans="1:8">
@@ -7432,7 +7432,7 @@
         <v>348.84907</v>
       </c>
       <c r="H175">
-        <v>782.23767</v>
+        <v>782.2376702</v>
       </c>
     </row>
     <row r="176" spans="1:8">
@@ -7458,7 +7458,7 @@
         <v>273.22687</v>
       </c>
       <c r="H176">
-        <v>491.24026</v>
+        <v>491.2402629</v>
       </c>
     </row>
     <row r="177" spans="1:8">
@@ -7484,7 +7484,7 @@
         <v>294.59593</v>
       </c>
       <c r="H177">
-        <v>597.94524</v>
+        <v>597.9452421</v>
       </c>
     </row>
     <row r="178" spans="1:8">
@@ -7510,7 +7510,7 @@
         <v>197.11105</v>
       </c>
       <c r="H178">
-        <v>461.348</v>
+        <v>461.3480017</v>
       </c>
     </row>
     <row r="179" spans="1:8">
@@ -7536,7 +7536,7 @@
         <v>331.98424</v>
       </c>
       <c r="H179">
-        <v>400.49525</v>
+        <v>400.4952459</v>
       </c>
     </row>
     <row r="180" spans="1:8">
@@ -7562,7 +7562,7 @@
         <v>293.17136</v>
       </c>
       <c r="H180">
-        <v>524.64709</v>
+        <v>524.6470859</v>
       </c>
     </row>
     <row r="181" spans="1:8">
@@ -7588,7 +7588,7 @@
         <v>479.95808</v>
       </c>
       <c r="H181">
-        <v>594.08371</v>
+        <v>594.0837125</v>
       </c>
     </row>
     <row r="182" spans="1:8">
@@ -7614,7 +7614,7 @@
         <v>364.92612</v>
       </c>
       <c r="H182">
-        <v>400.4454</v>
+        <v>400.4453993</v>
       </c>
     </row>
     <row r="183" spans="1:8">
@@ -7666,7 +7666,7 @@
         <v>563.0395</v>
       </c>
       <c r="H184">
-        <v>1131.26594</v>
+        <v>1131.265941</v>
       </c>
     </row>
     <row r="185" spans="1:8">
@@ -7692,7 +7692,7 @@
         <v>518.43562</v>
       </c>
       <c r="H185">
-        <v>921.1756800000001</v>
+        <v>921.1756812</v>
       </c>
     </row>
     <row r="186" spans="1:8">
@@ -7718,7 +7718,7 @@
         <v>514.90529</v>
       </c>
       <c r="H186">
-        <v>896.67832</v>
+        <v>896.6783158</v>
       </c>
     </row>
     <row r="187" spans="1:8">
@@ -7744,7 +7744,7 @@
         <v>521.93123</v>
       </c>
       <c r="H187">
-        <v>763.86631</v>
+        <v>763.8663129</v>
       </c>
     </row>
     <row r="188" spans="1:8">
@@ -7770,7 +7770,7 @@
         <v>577.51194</v>
       </c>
       <c r="H188">
-        <v>1207.13678</v>
+        <v>1207.136785</v>
       </c>
     </row>
     <row r="189" spans="1:8">
@@ -7796,7 +7796,7 @@
         <v>515.69795</v>
       </c>
       <c r="H189">
-        <v>648.6839</v>
+        <v>619.0867854000001</v>
       </c>
     </row>
     <row r="190" spans="1:8">
@@ -7822,7 +7822,7 @@
         <v>491.15339</v>
       </c>
       <c r="H190">
-        <v>576.58471</v>
+        <v>576.584713</v>
       </c>
     </row>
     <row r="191" spans="1:8">
@@ -7848,7 +7848,7 @@
         <v>435.01059</v>
       </c>
       <c r="H191">
-        <v>717.3635</v>
+        <v>717.3635035999999</v>
       </c>
     </row>
     <row r="192" spans="1:8">
@@ -7874,7 +7874,7 @@
         <v>284.59658</v>
       </c>
       <c r="H192">
-        <v>524.74665</v>
+        <v>524.7466454</v>
       </c>
     </row>
     <row r="193" spans="1:8">
@@ -7900,7 +7900,7 @@
         <v>113.15533</v>
       </c>
       <c r="H193">
-        <v>865.7155</v>
+        <v>865.7154998</v>
       </c>
     </row>
     <row r="194" spans="1:8">
@@ -7926,7 +7926,7 @@
         <v>264.31122</v>
       </c>
       <c r="H194">
-        <v>605.67007</v>
+        <v>605.6700724</v>
       </c>
     </row>
     <row r="195" spans="1:8">
@@ -7952,7 +7952,7 @@
         <v>652.47064</v>
       </c>
       <c r="H195">
-        <v>736.77854</v>
+        <v>736.7785431</v>
       </c>
     </row>
     <row r="196" spans="1:8">
@@ -7978,7 +7978,7 @@
         <v>573.80236</v>
       </c>
       <c r="H196">
-        <v>904.92785</v>
+        <v>904.9278519</v>
       </c>
     </row>
     <row r="197" spans="1:8">
@@ -8004,7 +8004,7 @@
         <v>462.05562</v>
       </c>
       <c r="H197">
-        <v>554.21192</v>
+        <v>554.2119218</v>
       </c>
     </row>
     <row r="198" spans="1:8">
@@ -8030,7 +8030,7 @@
         <v>40.8</v>
       </c>
       <c r="H198">
-        <v>527.45249</v>
+        <v>527.452492</v>
       </c>
     </row>
     <row r="199" spans="1:8">
@@ -8056,7 +8056,7 @@
         <v>304.17678</v>
       </c>
       <c r="H199">
-        <v>1091.88288</v>
+        <v>1091.882876</v>
       </c>
     </row>
     <row r="200" spans="1:8">
@@ -8082,7 +8082,7 @@
         <v>13.81251</v>
       </c>
       <c r="H200">
-        <v>193.01101</v>
+        <v>193.0110062</v>
       </c>
     </row>
     <row r="201" spans="1:8">
@@ -8108,7 +8108,7 @@
         <v>17.705</v>
       </c>
       <c r="H201">
-        <v>260.84704</v>
+        <v>260.847041</v>
       </c>
     </row>
     <row r="202" spans="1:8">
@@ -8134,7 +8134,7 @@
         <v>231.77998</v>
       </c>
       <c r="H202">
-        <v>736.59066</v>
+        <v>792.8366686000001</v>
       </c>
     </row>
     <row r="203" spans="1:8">
@@ -8160,7 +8160,7 @@
         <v>213.53292</v>
       </c>
       <c r="H203">
-        <v>899.66018</v>
+        <v>899.660176</v>
       </c>
     </row>
     <row r="204" spans="1:8">
@@ -8186,7 +8186,7 @@
         <v>287.43191</v>
       </c>
       <c r="H204">
-        <v>751.47304</v>
+        <v>751.4730382</v>
       </c>
     </row>
     <row r="205" spans="1:8">
@@ -8212,7 +8212,7 @@
         <v>154.44429</v>
       </c>
       <c r="H205">
-        <v>321.62406</v>
+        <v>321.624065</v>
       </c>
     </row>
     <row r="206" spans="1:8">
@@ -8238,7 +8238,7 @@
         <v>298.2481</v>
       </c>
       <c r="H206">
-        <v>804.73351</v>
+        <v>804.7335141999999</v>
       </c>
     </row>
     <row r="207" spans="1:8">
@@ -8264,7 +8264,7 @@
         <v>223.31487</v>
       </c>
       <c r="H207">
-        <v>382.43233</v>
+        <v>382.4323329</v>
       </c>
     </row>
     <row r="208" spans="1:8">
@@ -8290,7 +8290,7 @@
         <v>258.5688</v>
       </c>
       <c r="H208">
-        <v>700.43624</v>
+        <v>700.4362356</v>
       </c>
     </row>
     <row r="209" spans="1:8">
@@ -8316,7 +8316,7 @@
         <v>241.89922</v>
       </c>
       <c r="H209">
-        <v>655.15551</v>
+        <v>655.1555129</v>
       </c>
     </row>
     <row r="210" spans="1:8">
@@ -8342,7 +8342,7 @@
         <v>265.1549</v>
       </c>
       <c r="H210">
-        <v>405.74286</v>
+        <v>405.7428632</v>
       </c>
     </row>
     <row r="211" spans="1:8">
@@ -8368,7 +8368,7 @@
         <v>226.5732</v>
       </c>
       <c r="H211">
-        <v>384.14542</v>
+        <v>384.1454156</v>
       </c>
     </row>
     <row r="212" spans="1:8">
@@ -8394,7 +8394,7 @@
         <v>323.6479</v>
       </c>
       <c r="H212">
-        <v>808.3791</v>
+        <v>808.3791038000001</v>
       </c>
     </row>
     <row r="213" spans="1:8">
@@ -8420,7 +8420,7 @@
         <v>167.46908</v>
       </c>
       <c r="H213">
-        <v>340.01658</v>
+        <v>340.016583</v>
       </c>
     </row>
     <row r="214" spans="1:8">
@@ -8446,7 +8446,7 @@
         <v>235.50018</v>
       </c>
       <c r="H214">
-        <v>972.32393</v>
+        <v>972.3239334</v>
       </c>
     </row>
     <row r="215" spans="1:8">
@@ -8472,7 +8472,7 @@
         <v>234.40538</v>
       </c>
       <c r="H215">
-        <v>385.84617</v>
+        <v>385.8461735</v>
       </c>
     </row>
     <row r="216" spans="1:8">
@@ -8498,7 +8498,7 @@
         <v>287.826</v>
       </c>
       <c r="H216">
-        <v>745.73959</v>
+        <v>745.7395872</v>
       </c>
     </row>
     <row r="217" spans="1:8">
@@ -8524,7 +8524,7 @@
         <v>196.79213</v>
       </c>
       <c r="H217">
-        <v>367.04363</v>
+        <v>367.0436252</v>
       </c>
     </row>
     <row r="218" spans="1:8">
@@ -8550,7 +8550,7 @@
         <v>287.73547</v>
       </c>
       <c r="H218">
-        <v>752.80264</v>
+        <v>752.8026358</v>
       </c>
     </row>
     <row r="219" spans="1:8">
@@ -8576,7 +8576,7 @@
         <v>192.502</v>
       </c>
       <c r="H219">
-        <v>364.98872</v>
+        <v>364.9887246</v>
       </c>
     </row>
     <row r="220" spans="1:8">
@@ -8602,7 +8602,7 @@
         <v>154.35035</v>
       </c>
       <c r="H220">
-        <v>406.34587</v>
+        <v>406.3458744</v>
       </c>
     </row>
     <row r="221" spans="1:8">
@@ -8628,7 +8628,7 @@
         <v>161.47656</v>
       </c>
       <c r="H221">
-        <v>478.49264</v>
+        <v>478.4926371</v>
       </c>
     </row>
     <row r="222" spans="1:8">
@@ -8654,7 +8654,7 @@
         <v>313.08768</v>
       </c>
       <c r="H222">
-        <v>393.84914</v>
+        <v>393.8491419</v>
       </c>
     </row>
     <row r="223" spans="1:8">
@@ -8680,7 +8680,7 @@
         <v>248.02501</v>
       </c>
       <c r="H223">
-        <v>460.31701</v>
+        <v>460.3170135</v>
       </c>
     </row>
     <row r="224" spans="1:8">
@@ -8706,7 +8706,7 @@
         <v>266.20541</v>
       </c>
       <c r="H224">
-        <v>701.29465</v>
+        <v>701.2946469</v>
       </c>
     </row>
     <row r="225" spans="1:8">
@@ -8732,7 +8732,7 @@
         <v>204.80692</v>
       </c>
       <c r="H225">
-        <v>371.62297</v>
+        <v>371.6229696</v>
       </c>
     </row>
     <row r="226" spans="1:8">
@@ -8758,7 +8758,7 @@
         <v>330.39045</v>
       </c>
       <c r="H226">
-        <v>669.75458</v>
+        <v>669.7545778</v>
       </c>
     </row>
     <row r="227" spans="1:8">
@@ -8784,7 +8784,7 @@
         <v>264.56716</v>
       </c>
       <c r="H227">
-        <v>851.15535</v>
+        <v>851.1553453</v>
       </c>
     </row>
     <row r="228" spans="1:8">
@@ -8810,7 +8810,7 @@
         <v>231.87628</v>
       </c>
       <c r="H228">
-        <v>386.55504</v>
+        <v>386.5550398</v>
       </c>
     </row>
     <row r="229" spans="1:8">
@@ -8836,7 +8836,7 @@
         <v>222.21164</v>
       </c>
       <c r="H229">
-        <v>414.98917</v>
+        <v>414.9891702</v>
       </c>
     </row>
     <row r="230" spans="1:8">
@@ -8862,7 +8862,7 @@
         <v>227.73894</v>
       </c>
       <c r="H230">
-        <v>616.14198</v>
+        <v>616.1419793</v>
       </c>
     </row>
     <row r="231" spans="1:8">
@@ -8888,7 +8888,7 @@
         <v>221.85461</v>
       </c>
       <c r="H231">
-        <v>378.09544</v>
+        <v>378.0954361</v>
       </c>
     </row>
     <row r="232" spans="1:8">
@@ -8914,7 +8914,7 @@
         <v>450.34825</v>
       </c>
       <c r="H232">
-        <v>1036.9368</v>
+        <v>1036.936803</v>
       </c>
     </row>
     <row r="233" spans="1:8">
@@ -8940,7 +8940,7 @@
         <v>442.70108</v>
       </c>
       <c r="H233">
-        <v>1347.94853</v>
+        <v>1347.948526</v>
       </c>
     </row>
     <row r="234" spans="1:8">
@@ -8966,7 +8966,7 @@
         <v>285.0211</v>
       </c>
       <c r="H234">
-        <v>467.81658</v>
+        <v>467.816584</v>
       </c>
     </row>
     <row r="235" spans="1:8">
@@ -8992,7 +8992,7 @@
         <v>437.5176</v>
       </c>
       <c r="H235">
-        <v>914.71488</v>
+        <v>914.7148794</v>
       </c>
     </row>
     <row r="236" spans="1:8">

</xml_diff>